<commit_message>
Add board_M to pegs_M_150mm
board_M.stl is the FMB peg board whose holes fit the size-M pegs.
index.csv gains its row; index.xlsx gets a part column and a Summary
split into all files / pegs / board, so peg statistics are not mixed
with the board. Ignore Office lock files.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pegs_M_150mm/index.xlsx
+++ b/pegs_M_150mm/index.xlsx
@@ -94,7 +94,7 @@
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -465,34 +465,35 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="68" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="68" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>FMB pegs, size M, length 150 mm</t>
+          <t>FMB size M: 9 pegs, length 150 mm, and board_M.stl</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Measured from the STL files in this folder by make_index.py. index.csv has the same measurements (rounded) plus units, scale_to_mm, source, changes and license, which are in the Summary notes here.</t>
+          <t>Measured from the STL files in this folder by make_index.py (part and shape are read from the file name). index.csv has the same measurements (rounded) plus units, scale_to_mm, source, changes and license, which are in the Summary notes here.</t>
         </is>
       </c>
     </row>
@@ -504,55 +505,60 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
+          <t>part</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
           <t>shape</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>size_bytes</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>size_MB</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>stl_format</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>triangles</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>x_mm</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>y_mm</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>z_mm</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>volume_cm3</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>watertight</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>sha256</t>
         </is>
@@ -561,449 +567,542 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>peg_arch_M_150mm.stl</t>
+          <t>board_M.stl</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>arch</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="n">
-        <v>96684</v>
-      </c>
-      <c r="D5" s="5">
-        <f>C5/1000000</f>
-        <v>0.096684</v>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
+          <t>board</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="4" t="n">
+        <v>1447384</v>
+      </c>
+      <c r="E5" s="5">
+        <f>D5/1000000</f>
+        <v>1.447384</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>binary</t>
         </is>
       </c>
-      <c r="F5" s="4" t="n">
-        <v>1932</v>
-      </c>
-      <c r="G5" s="6" t="n">
-        <v>48</v>
+      <c r="G5" s="4" t="n">
+        <v>28946</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>28.79999542236328</v>
+        <v>230</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>150</v>
-      </c>
-      <c r="J5" s="7" t="n">
-        <v>150.2945201516733</v>
-      </c>
-      <c r="K5" s="2" t="b">
+        <v>230</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="K5" s="7" t="n">
+        <v>2123.111080751493</v>
+      </c>
+      <c r="L5" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>356414eed62620ed0576f65938d6103c73f98a8f0c58055adee88ee360124bae</t>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>de88ec19bfd098f37496a539359e875308e41408d593c555f1076eee9a20ae67</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>peg_circle_M_150mm.stl</t>
+          <t>peg_arch_M_150mm.stl</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>circle</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>50284</v>
-      </c>
-      <c r="D6" s="5">
-        <f>C6/1000000</f>
-        <v>0.050284</v>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
+          <t>peg</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>arch</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>96684</v>
+      </c>
+      <c r="E6" s="5">
+        <f>D6/1000000</f>
+        <v>0.096684</v>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>binary</t>
         </is>
       </c>
-      <c r="F6" s="4" t="n">
-        <v>1004</v>
-      </c>
-      <c r="G6" s="6" t="n">
-        <v>40.31997680664062</v>
+      <c r="G6" s="4" t="n">
+        <v>1932</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>40.31999969482422</v>
+        <v>48</v>
       </c>
       <c r="I6" s="6" t="n">
+        <v>28.79999542236328</v>
+      </c>
+      <c r="J6" s="6" t="n">
         <v>150</v>
       </c>
-      <c r="J6" s="7" t="n">
-        <v>191.5036946361564</v>
-      </c>
-      <c r="K6" s="2" t="b">
+      <c r="K6" s="7" t="n">
+        <v>150.2945201516733</v>
+      </c>
+      <c r="L6" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>73b154b575860f7094ee534145bc112b60533f967a92f8ebb3fa229e2546a55e</t>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>356414eed62620ed0576f65938d6103c73f98a8f0c58055adee88ee360124bae</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>peg_double_square_M_150mm.stl</t>
+          <t>peg_circle_M_150mm.stl</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>double_square</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="n">
-        <v>102284</v>
-      </c>
-      <c r="D7" s="5">
-        <f>C7/1000000</f>
-        <v>0.102284</v>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
+          <t>peg</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>circle</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>50284</v>
+      </c>
+      <c r="E7" s="5">
+        <f>D7/1000000</f>
+        <v>0.050284</v>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>binary</t>
         </is>
       </c>
-      <c r="F7" s="4" t="n">
-        <v>2044</v>
-      </c>
-      <c r="G7" s="6" t="n">
-        <v>53.00189208984375</v>
+      <c r="G7" s="4" t="n">
+        <v>1004</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>20.38533782958984</v>
+        <v>40.31997680664062</v>
       </c>
       <c r="I7" s="6" t="n">
+        <v>40.31999969482422</v>
+      </c>
+      <c r="J7" s="6" t="n">
         <v>150</v>
       </c>
-      <c r="J7" s="7" t="n">
-        <v>142.2127081230414</v>
-      </c>
-      <c r="K7" s="2" t="b">
+      <c r="K7" s="7" t="n">
+        <v>191.5036946361564</v>
+      </c>
+      <c r="L7" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>0971753d95f52c3600dbe33fbd44a8f834015dd6d349983787b3af02374b0fb8</t>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>73b154b575860f7094ee534145bc112b60533f967a92f8ebb3fa229e2546a55e</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>peg_ellipse_M_150mm.stl</t>
+          <t>peg_double_square_M_150mm.stl</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>ellipse</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="n">
-        <v>66284</v>
-      </c>
-      <c r="D8" s="5">
-        <f>C8/1000000</f>
-        <v>0.066284</v>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
+          <t>peg</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>double_square</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>102284</v>
+      </c>
+      <c r="E8" s="5">
+        <f>D8/1000000</f>
+        <v>0.102284</v>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>binary</t>
         </is>
       </c>
-      <c r="F8" s="4" t="n">
-        <v>1324</v>
-      </c>
-      <c r="G8" s="6" t="n">
-        <v>43.19989013671875</v>
+      <c r="G8" s="4" t="n">
+        <v>2044</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>28.79920959472656</v>
+        <v>53.00189208984375</v>
       </c>
       <c r="I8" s="6" t="n">
+        <v>20.38533782958984</v>
+      </c>
+      <c r="J8" s="6" t="n">
         <v>150</v>
       </c>
-      <c r="J8" s="7" t="n">
-        <v>146.5643927405588</v>
-      </c>
-      <c r="K8" s="2" t="b">
+      <c r="K8" s="7" t="n">
+        <v>142.2127081230414</v>
+      </c>
+      <c r="L8" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>fc9e6bbefa53817214ea440a3b8a1cb8bfca0dc51ff69ad9dfc9685abb24f3b8</t>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>0971753d95f52c3600dbe33fbd44a8f834015dd6d349983787b3af02374b0fb8</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>peg_hexagon_M_150mm.stl</t>
+          <t>peg_ellipse_M_150mm.stl</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>hexagon</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="n">
-        <v>51484</v>
-      </c>
-      <c r="D9" s="5">
-        <f>C9/1000000</f>
-        <v>0.051484</v>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
+          <t>peg</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>ellipse</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>66284</v>
+      </c>
+      <c r="E9" s="5">
+        <f>D9/1000000</f>
+        <v>0.066284</v>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>binary</t>
         </is>
       </c>
-      <c r="F9" s="4" t="n">
-        <v>1028</v>
-      </c>
-      <c r="G9" s="6" t="n">
-        <v>36.5809326171875</v>
+      <c r="G9" s="4" t="n">
+        <v>1324</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>41.34892272949219</v>
+        <v>43.19989013671875</v>
       </c>
       <c r="I9" s="6" t="n">
+        <v>28.79920959472656</v>
+      </c>
+      <c r="J9" s="6" t="n">
         <v>150</v>
       </c>
-      <c r="J9" s="7" t="n">
-        <v>173.4309555758955</v>
-      </c>
-      <c r="K9" s="2" t="b">
+      <c r="K9" s="7" t="n">
+        <v>146.5643927405588</v>
+      </c>
+      <c r="L9" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>98d141f3666dc5548d7bfab7e383c4a75d7c188fad4bc267ae3599c34bdb4b5f</t>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>fc9e6bbefa53817214ea440a3b8a1cb8bfca0dc51ff69ad9dfc9685abb24f3b8</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>peg_rectangle_M_150mm.stl</t>
+          <t>peg_hexagon_M_150mm.stl</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>rectangle</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="n">
-        <v>51084</v>
-      </c>
-      <c r="D10" s="5">
-        <f>C10/1000000</f>
-        <v>0.051084</v>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
+          <t>peg</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>hexagon</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>51484</v>
+      </c>
+      <c r="E10" s="5">
+        <f>D10/1000000</f>
+        <v>0.051484</v>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>binary</t>
         </is>
       </c>
-      <c r="F10" s="4" t="n">
-        <v>1020</v>
-      </c>
-      <c r="G10" s="6" t="n">
-        <v>40.32000732421875</v>
+      <c r="G10" s="4" t="n">
+        <v>1028</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>25.92000579833984</v>
+        <v>36.5809326171875</v>
       </c>
       <c r="I10" s="6" t="n">
+        <v>41.34892272949219</v>
+      </c>
+      <c r="J10" s="6" t="n">
         <v>150</v>
       </c>
-      <c r="J10" s="7" t="n">
-        <v>155.6958128524711</v>
-      </c>
-      <c r="K10" s="2" t="b">
+      <c r="K10" s="7" t="n">
+        <v>173.4309555758955</v>
+      </c>
+      <c r="L10" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>f9baf06ae2aa28748dbccc68564021042ef96e2df30e82cd7e5d97b356623874</t>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>98d141f3666dc5548d7bfab7e383c4a75d7c188fad4bc267ae3599c34bdb4b5f</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>peg_square_round_M_150mm.stl</t>
+          <t>peg_rectangle_M_150mm.stl</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>square_round</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="n">
-        <v>101684</v>
-      </c>
-      <c r="D11" s="5">
-        <f>C11/1000000</f>
-        <v>0.101684</v>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
+          <t>peg</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>rectangle</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>51084</v>
+      </c>
+      <c r="E11" s="5">
+        <f>D11/1000000</f>
+        <v>0.051084</v>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>binary</t>
         </is>
       </c>
-      <c r="F11" s="4" t="n">
-        <v>2032</v>
-      </c>
-      <c r="G11" s="6" t="n">
-        <v>52.79998779296875</v>
+      <c r="G11" s="4" t="n">
+        <v>1020</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>19.80001068115234</v>
+        <v>40.32000732421875</v>
       </c>
       <c r="I11" s="6" t="n">
+        <v>25.92000579833984</v>
+      </c>
+      <c r="J11" s="6" t="n">
         <v>150</v>
       </c>
-      <c r="J11" s="7" t="n">
-        <v>126.2305741329241</v>
-      </c>
-      <c r="K11" s="2" t="b">
+      <c r="K11" s="7" t="n">
+        <v>155.6958128524711</v>
+      </c>
+      <c r="L11" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
-          <t>8f571bf08a1a6c3227cc142fb493cf4b334c3b92146c9d4ed2e5264e37fcf50f</t>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>f9baf06ae2aa28748dbccc68564021042ef96e2df30e82cd7e5d97b356623874</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>peg_star_M_150mm.stl</t>
+          <t>peg_square_round_M_150mm.stl</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>star</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="n">
-        <v>102884</v>
-      </c>
-      <c r="D12" s="5">
-        <f>C12/1000000</f>
-        <v>0.102884</v>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
+          <t>peg</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>square_round</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>101684</v>
+      </c>
+      <c r="E12" s="5">
+        <f>D12/1000000</f>
+        <v>0.101684</v>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>binary</t>
         </is>
       </c>
-      <c r="F12" s="4" t="n">
-        <v>2056</v>
-      </c>
-      <c r="G12" s="6" t="n">
-        <v>43.95175170898438</v>
+      <c r="G12" s="4" t="n">
+        <v>2032</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>42.082275390625</v>
+        <v>52.79998779296875</v>
       </c>
       <c r="I12" s="6" t="n">
+        <v>19.80001068115234</v>
+      </c>
+      <c r="J12" s="6" t="n">
         <v>150</v>
       </c>
-      <c r="J12" s="7" t="n">
-        <v>134.2015609002323</v>
-      </c>
-      <c r="K12" s="2" t="b">
+      <c r="K12" s="7" t="n">
+        <v>126.2305741329241</v>
+      </c>
+      <c r="L12" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>095f06b95f64337f83cb12a974f85f51ab0ed4680db3501a33c446907f718e1f</t>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>8f571bf08a1a6c3227cc142fb493cf4b334c3b92146c9d4ed2e5264e37fcf50f</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
+          <t>peg_star_M_150mm.stl</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>peg</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>star</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>102884</v>
+      </c>
+      <c r="E13" s="5">
+        <f>D13/1000000</f>
+        <v>0.102884</v>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>2056</v>
+      </c>
+      <c r="H13" s="6" t="n">
+        <v>43.95175170898438</v>
+      </c>
+      <c r="I13" s="6" t="n">
+        <v>42.082275390625</v>
+      </c>
+      <c r="J13" s="6" t="n">
+        <v>150</v>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>134.2015609002323</v>
+      </c>
+      <c r="L13" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>095f06b95f64337f83cb12a974f85f51ab0ed4680db3501a33c446907f718e1f</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
           <t>peg_three_prong_M_150mm.stl</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>peg</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>three_prong</t>
         </is>
       </c>
-      <c r="C13" s="4" t="n">
+      <c r="D14" s="4" t="n">
         <v>304884</v>
       </c>
-      <c r="D13" s="5">
-        <f>C13/1000000</f>
+      <c r="E14" s="5">
+        <f>D14/1000000</f>
         <v>0.304884</v>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>binary</t>
         </is>
       </c>
-      <c r="F13" s="4" t="n">
+      <c r="G14" s="4" t="n">
         <v>6096</v>
       </c>
-      <c r="G13" s="6" t="n">
+      <c r="H14" s="6" t="n">
         <v>52.79998779296875</v>
       </c>
-      <c r="H13" s="6" t="n">
+      <c r="I14" s="6" t="n">
         <v>49.26306915283203</v>
       </c>
-      <c r="I13" s="6" t="n">
+      <c r="J14" s="6" t="n">
         <v>150</v>
       </c>
-      <c r="J13" s="7" t="n">
+      <c r="K14" s="7" t="n">
         <v>151.2762522948021</v>
       </c>
-      <c r="K13" s="2" t="b">
+      <c r="L14" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="M14" s="2" t="inlineStr">
         <is>
           <t>af83d8e0f5d8269afaa408f4a5ab448f07c9633ffbdc7a8e20ba3eacaf324096</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C14" s="9">
-        <f>SUM(C5:C13)</f>
-        <v>927556</v>
-      </c>
-      <c r="D14" s="10">
-        <f>C14/1000000</f>
-        <v>0.927556</v>
-      </c>
-      <c r="F14" s="9">
-        <f>SUM(F5:F13)</f>
-        <v>18536</v>
-      </c>
-      <c r="J14" s="11">
-        <f>SUM(J5:J13)</f>
-        <v>1371.410471407755</v>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="D15" s="9">
+        <f>SUM(D5:D14)</f>
+        <v>2374940</v>
+      </c>
+      <c r="E15" s="10">
+        <f>D15/1000000</f>
+        <v>2.37494</v>
+      </c>
+      <c r="G15" s="9">
+        <f>SUM(G5:G14)</f>
+        <v>47482</v>
+      </c>
+      <c r="K15" s="11">
+        <f>SUM(K5:K14)</f>
+        <v>3494.5215521592477</v>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>(watertight parts)</t>
         </is>
@@ -1020,7 +1119,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1031,7 +1130,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Summary: FMB pegs, size M, length 150 mm</t>
+          <t>Summary: FMB size M: 9 pegs, length 150 mm, and board_M.stl</t>
         </is>
       </c>
     </row>
@@ -1053,44 +1152,35 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>files</t>
-        </is>
-      </c>
-      <c r="B4" s="12">
-        <f>COUNTA(Files!A5:A13)</f>
-        <v>9</v>
-      </c>
-      <c r="C4" s="2" t="inlineStr"/>
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>All files</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>watertight files</t>
+          <t>files</t>
         </is>
       </c>
       <c r="B5" s="12">
-        <f>COUNTIF(Files!K5:K13,TRUE)</f>
-        <v>9</v>
+        <f>COUNTA(Files!A5:A14)</f>
+        <v>10</v>
       </c>
       <c r="C5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>total size</t>
-        </is>
-      </c>
-      <c r="B6" s="13">
-        <f>SUM(Files!C5:C13)</f>
-        <v>927556</v>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>bytes</t>
-        </is>
-      </c>
+          <t>watertight files</t>
+        </is>
+      </c>
+      <c r="B6" s="12">
+        <f>COUNTIF(Files!L5:L14,TRUE)</f>
+        <v>10</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1098,53 +1188,53 @@
           <t>total size</t>
         </is>
       </c>
-      <c r="B7" s="14">
-        <f>SUM(Files!C5:C13)/1000000</f>
-        <v>0.927556</v>
+      <c r="B7" s="13">
+        <f>SUM(Files!D5:D14)</f>
+        <v>2374940</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>MB (1e6 bytes)</t>
+          <t>bytes</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>total triangles</t>
-        </is>
-      </c>
-      <c r="B8" s="13">
-        <f>SUM(Files!F5:F13)</f>
-        <v>18536</v>
-      </c>
-      <c r="C8" s="2" t="inlineStr"/>
+          <t>total size</t>
+        </is>
+      </c>
+      <c r="B8" s="14">
+        <f>SUM(Files!D5:D14)/1000000</f>
+        <v>2.37494</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>MB (1e6 bytes)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>total volume (watertight parts)</t>
-        </is>
-      </c>
-      <c r="B9" s="15">
-        <f>SUM(Files!J5:J13)</f>
-        <v>1371.410471407755</v>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>cm3</t>
-        </is>
-      </c>
+          <t>total triangles</t>
+        </is>
+      </c>
+      <c r="B9" s="13">
+        <f>SUM(Files!G5:G14)</f>
+        <v>47482</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>mean volume (watertight parts)</t>
+          <t>total volume (watertight parts)</t>
         </is>
       </c>
       <c r="B10" s="15">
-        <f>AVERAGE(Files!J5:J13)</f>
-        <v>152.37894126752835</v>
+        <f>SUM(Files!K5:K14)</f>
+        <v>3494.5215521592477</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -1155,209 +1245,355 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>min volume (watertight parts)</t>
-        </is>
-      </c>
-      <c r="B11" s="15">
-        <f>MIN(Files!J5:J13)</f>
-        <v>126.2305741329241</v>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>cm3</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>max volume (watertight parts)</t>
-        </is>
-      </c>
-      <c r="B12" s="15">
-        <f>MAX(Files!J5:J13)</f>
-        <v>191.5036946361564</v>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>cm3</t>
-        </is>
-      </c>
+          <t>largest file</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="str">
+        <f>INDEX(Files!A5:A14,MATCH(MAX(Files!D5:D14),Files!D5:D14,0))</f>
+        <v>board_M.stl</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>largest volume part</t>
-        </is>
-      </c>
-      <c r="B13" s="16" t="str">
-        <f>INDEX(Files!A5:A13,MATCH(MAX(Files!J5:J13),Files!J5:J13,0))</f>
-        <v>peg_circle_M_150mm.stl</v>
-      </c>
-      <c r="C13" s="2" t="inlineStr"/>
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Pegs</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>largest file</t>
-        </is>
-      </c>
-      <c r="B14" s="16" t="str">
-        <f>INDEX(Files!A5:A13,MATCH(MAX(Files!C5:C13),Files!C5:C13,0))</f>
-        <v>peg_three_prong_M_150mm.stl</v>
+          <t>pegs</t>
+        </is>
+      </c>
+      <c r="B14" s="12">
+        <f>COUNTA(Files!A6:A14)</f>
+        <v>9</v>
       </c>
       <c r="C14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>max x (footprint)</t>
-        </is>
-      </c>
-      <c r="B15" s="17">
-        <f>MAX(Files!G5:G13)</f>
-        <v>53.00189208984375</v>
+          <t>total volume (watertight pegs)</t>
+        </is>
+      </c>
+      <c r="B15" s="15">
+        <f>SUM(Files!K6:K14)</f>
+        <v>1371.410471407755</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>cm3</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>max y (footprint)</t>
-        </is>
-      </c>
-      <c r="B16" s="17">
-        <f>MAX(Files!H5:H13)</f>
-        <v>49.26306915283203</v>
+          <t>mean volume (watertight pegs)</t>
+        </is>
+      </c>
+      <c r="B16" s="15">
+        <f>AVERAGE(Files!K6:K14)</f>
+        <v>152.37894126752835</v>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>cm3</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>min z (height)</t>
-        </is>
-      </c>
-      <c r="B17" s="17">
-        <f>MIN(Files!I5:I13)</f>
-        <v>150.0</v>
+          <t>min volume (watertight pegs)</t>
+        </is>
+      </c>
+      <c r="B17" s="15">
+        <f>MIN(Files!K6:K14)</f>
+        <v>126.2305741329241</v>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>cm3</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>max z (height)</t>
-        </is>
-      </c>
-      <c r="B18" s="17">
-        <f>MAX(Files!I5:I13)</f>
-        <v>150.0</v>
+          <t>max volume (watertight pegs)</t>
+        </is>
+      </c>
+      <c r="B18" s="15">
+        <f>MAX(Files!K6:K14)</f>
+        <v>191.5036946361564</v>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
+          <t>cm3</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>largest volume peg</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="str">
+        <f>INDEX(Files!A6:A14,MATCH(MAX(Files!K6:K14),Files!K6:K14,0))</f>
+        <v>peg_circle_M_150mm.stl</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>max x (footprint)</t>
+        </is>
+      </c>
+      <c r="B20" s="17">
+        <f>MAX(Files!H6:H14)</f>
+        <v>53.00189208984375</v>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
           <t>mm</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
-        <is>
-          <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>units</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>mm (STL coordinates, scale_to_mm = 1); x/y/z = axis-aligned bounding box in the file's own orientation</t>
+          <t>max y (footprint)</t>
+        </is>
+      </c>
+      <c r="B21" s="17">
+        <f>MAX(Files!I6:I14)</f>
+        <v>49.26306915283203</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>mm</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>volume_cm3</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>enclosed solid volume of the mesh, blank if not watertight; printed mass also depends on infill and walls</t>
+          <t>min z (length)</t>
+        </is>
+      </c>
+      <c r="B22" s="17">
+        <f>MIN(Files!J6:J14)</f>
+        <v>150.0</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>mm</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>size_MB</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>size_bytes / 1e6 (decimal MB, not MiB)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>sha256</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>SHA-256 of the file bytes</t>
+          <t>max z (length)</t>
+        </is>
+      </c>
+      <c r="B23" s="17">
+        <f>MAX(Files!J6:J14)</f>
+        <v>150.0</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>mm</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>source</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>FMB (Luo et al.), peg.step, listed at https://functional-manipulation-benchmark.github.io/files/</t>
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>Board</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>changes</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>STEP solid tessellated to STL (linear deflection 0.01 relative to edge size, angular 0.05 rad); translated so XY bbox centre = origin and min z = 0; not rotated</t>
-        </is>
-      </c>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="B26" s="16" t="str">
+        <f>Files!A5</f>
+        <v>board_M.stl</v>
+      </c>
+      <c r="C26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
+          <t>x (bounding box)</t>
+        </is>
+      </c>
+      <c r="B27" s="17">
+        <f>Files!H5</f>
+        <v>230.0</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>y (bounding box)</t>
+        </is>
+      </c>
+      <c r="B28" s="17">
+        <f>Files!I5</f>
+        <v>230.0</v>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>z (bounding box)</t>
+        </is>
+      </c>
+      <c r="B29" s="17">
+        <f>Files!J5</f>
+        <v>50.0</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>volume</t>
+        </is>
+      </c>
+      <c r="B30" s="15">
+        <f>Files!K5</f>
+        <v>2123.111080751493</v>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>cm3</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>mm (STL coordinates, scale_to_mm = 1); x/y/z = axis-aligned bounding box in the file's own orientation</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>volume_cm3</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>enclosed solid volume of the mesh, blank if not watertight; printed mass also depends on infill and walls</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>size_MB</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>size_bytes / 1e6 (decimal MB, not MiB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>sha256</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>SHA-256 of the file bytes</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>source, pegs</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>FMB (Luo et al.), peg.step, listed at https://functional-manipulation-benchmark.github.io/files/</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>source, board</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>FMB (Luo et al.), peg_board.step, listed at https://functional-manipulation-benchmark.github.io/files/</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>changes</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>STEP solid tessellated to STL (linear deflection 0.01 relative to edge size, angular 0.05 rad); translated so XY bbox centre = origin and min z = 0; not rotated</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
           <t>license</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>CC BY 4.0, https://creativecommons.org/licenses/by/4.0/</t>
         </is>

</xml_diff>